<commit_message>
Cleaned up obsolete design files
</commit_message>
<xml_diff>
--- a/Documentation/Experiments/Joint Section Test Prints_no_travel.xlsx
+++ b/Documentation/Experiments/Joint Section Test Prints_no_travel.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucas\Documents\Projects\Co_Printing\Documentation\Experiments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EC6CDF7-EA12-4CB5-9A66-97EB6E6D118B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15F411E0-8590-481B-B4D9-4B7A77BA1332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17790" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,18 +36,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="12">
   <si>
     <t>Layer height</t>
   </si>
   <si>
     <t>Travel Length</t>
-  </si>
-  <si>
-    <t>Base Parameters</t>
-  </si>
-  <si>
-    <t>Nozzle Distance / mm</t>
   </si>
   <si>
     <t>Travel Speed / mm/s</t>
@@ -57,12 +51,6 @@
 Total Length</t>
   </si>
   <si>
-    <t>0/2</t>
-  </si>
-  <si>
-    <t>1/2</t>
-  </si>
-  <si>
     <t>Layer deposition interval / s   at distance x mm</t>
   </si>
   <si>
@@ -76,6 +64,15 @@
   </si>
   <si>
     <t>(150-2X)/C2</t>
+  </si>
+  <si>
+    <t>2/2</t>
+  </si>
+  <si>
+    <t>Boundry Joining Interval / s</t>
+  </si>
+  <si>
+    <t>To next material</t>
   </si>
 </sst>
 </file>
@@ -155,7 +152,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -183,6 +180,13 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -192,7 +196,9 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -388,7 +394,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V14"/>
+  <sheetPr codeName="Sheet1"/>
+  <dimension ref="A1:V16"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="14" width="11.5703125" style="2"/>
@@ -402,7 +409,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C2" s="3">
         <v>5</v>
@@ -443,18 +450,14 @@
       <c r="P2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="T2" s="5" t="s">
+      <c r="T2" s="5"/>
+      <c r="U2" s="5"/>
+      <c r="V2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="U2" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="V2" s="5" t="s">
-        <v>4</v>
-      </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A3" s="11">
+      <c r="A3" s="14">
         <v>0.3</v>
       </c>
       <c r="B3" s="6">
@@ -472,20 +475,13 @@
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
       <c r="N3" s="7"/>
-      <c r="P3" s="4">
-        <f>B3/2</f>
-        <v>25</v>
-      </c>
-      <c r="U3" s="2">
-        <f>P3</f>
-        <v>25</v>
-      </c>
+      <c r="P3" s="4"/>
       <c r="V3" s="2">
         <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A4" s="11"/>
+      <c r="A4" s="14"/>
       <c r="B4" s="6">
         <v>100</v>
       </c>
@@ -501,43 +497,51 @@
       <c r="L4" s="7"/>
       <c r="M4" s="7"/>
       <c r="N4" s="7"/>
-      <c r="P4" s="4">
-        <f>B4/2</f>
-        <v>50</v>
-      </c>
-      <c r="U4" s="2">
-        <f>P4</f>
-        <v>50</v>
-      </c>
+      <c r="P4" s="4"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A5" s="11"/>
+      <c r="A5" s="14"/>
       <c r="B5" s="6">
         <v>150</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
-      <c r="K5" s="7"/>
-      <c r="L5" s="7"/>
-      <c r="M5" s="7"/>
+        <v>9</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="M5" s="7" t="s">
+        <v>9</v>
+      </c>
       <c r="N5" s="7" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="P5" s="4">
-        <f>B5/2</f>
-        <v>75</v>
-      </c>
-      <c r="U5" s="2">
-        <f>P5</f>
-        <v>75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.2"/>
@@ -576,10 +580,10 @@
       <c r="O8"/>
     </row>
     <row r="9" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="13"/>
+      <c r="A9" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="16"/>
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
       <c r="E9" s="8"/>
@@ -595,8 +599,8 @@
       <c r="O9" s="9"/>
     </row>
     <row r="10" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="12"/>
-      <c r="B10" s="13"/>
+      <c r="A10" s="15"/>
+      <c r="B10" s="16"/>
       <c r="C10" s="8"/>
       <c r="D10" s="8"/>
       <c r="E10" s="8"/>
@@ -612,8 +616,8 @@
       <c r="O10" s="9"/>
     </row>
     <row r="11" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="12"/>
-      <c r="B11" s="13"/>
+      <c r="A11" s="15"/>
+      <c r="B11" s="16"/>
       <c r="C11" s="8"/>
       <c r="D11" s="8"/>
       <c r="E11" s="8"/>
@@ -629,8 +633,8 @@
       <c r="O11" s="9"/>
     </row>
     <row r="12" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="12"/>
-      <c r="B12" s="13"/>
+      <c r="A12" s="15"/>
+      <c r="B12" s="16"/>
       <c r="C12" s="8"/>
       <c r="D12" s="8"/>
       <c r="E12" s="8"/>
@@ -646,12 +650,12 @@
       <c r="O12" s="9"/>
     </row>
     <row r="13" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="12"/>
-      <c r="B13" s="13">
+      <c r="A13" s="15"/>
+      <c r="B13" s="16">
         <v>150</v>
       </c>
-      <c r="C13" s="14" t="s">
-        <v>11</v>
+      <c r="C13" s="13" t="s">
+        <v>7</v>
       </c>
       <c r="D13" s="8"/>
       <c r="E13" s="8"/>
@@ -665,14 +669,14 @@
       <c r="M13" s="8"/>
       <c r="N13" s="8"/>
       <c r="O13" s="9" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="12"/>
-      <c r="B14" s="13"/>
+      <c r="A14" s="15"/>
+      <c r="B14" s="16"/>
       <c r="C14" s="10" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D14" s="10"/>
       <c r="E14" s="10"/>
@@ -686,7 +690,66 @@
       <c r="M14" s="10"/>
       <c r="N14" s="10"/>
       <c r="O14" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="11" t="s">
         <v>10</v>
+      </c>
+      <c r="B16" s="12">
+        <v>150</v>
+      </c>
+      <c r="C16" s="17">
+        <f>75/C2</f>
+        <v>15</v>
+      </c>
+      <c r="D16" s="17">
+        <f t="shared" ref="D16:N16" si="0">75/D2</f>
+        <v>7.5</v>
+      </c>
+      <c r="E16" s="17">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="F16" s="17">
+        <f t="shared" si="0"/>
+        <v>3.75</v>
+      </c>
+      <c r="G16" s="17">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H16" s="17">
+        <f t="shared" si="0"/>
+        <v>2.5</v>
+      </c>
+      <c r="I16" s="17">
+        <f t="shared" si="0"/>
+        <v>2.1428571428571428</v>
+      </c>
+      <c r="J16" s="17">
+        <f t="shared" si="0"/>
+        <v>1.875</v>
+      </c>
+      <c r="K16" s="17">
+        <f t="shared" si="0"/>
+        <v>1.6666666666666667</v>
+      </c>
+      <c r="L16" s="17">
+        <f t="shared" si="0"/>
+        <v>1.5</v>
+      </c>
+      <c r="M16" s="17">
+        <f t="shared" si="0"/>
+        <v>1.3636363636363635</v>
+      </c>
+      <c r="N16" s="17">
+        <f t="shared" si="0"/>
+        <v>1.25</v>
+      </c>
+      <c r="O16" s="11" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>